<commit_message>
XL: Saharsh locks 8 rows, fix rows 20/21 Ch refs
Assisted-by: Muse Spark (opencode)
</commit_message>
<xml_diff>
--- a/docs/report/Chapter2_40_papers.xlsx
+++ b/docs/report/Chapter2_40_papers.xlsx
@@ -902,82 +902,82 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>[2]</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Intrusion detection systems: A survey and taxonomy</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>S. Axelsson</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Chalmers Tech. Rep. 99-15, 2000</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>http://citeseerx.ist.psu.edu/viewdoc/summary?doi=10.1.1.1.6603</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>[3]</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Anomaly detection: A survey</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>V. Chandola, A. Banerjee, V. Kumar</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>ACM Comput. Surv. 41(3), 2009</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/1541880.1541882</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
@@ -1022,42 +1022,42 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>[5]</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Toward generating a new intrusion detection dataset and intrusion traffic characterization (CICIDS2017)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>I. Sharafaldin, A. H. Lashkari, A. A. Ghorbani</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>ICISSP 2018</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>https://doi.org/10.5220/0006639801080116</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
@@ -1182,42 +1182,42 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>[9]</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>CICFlowMeter (flow feature extractor)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>A. H. Lashkari / CIC</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>https://github.com/ahlashkari/CICFlowMeter</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
@@ -1262,42 +1262,42 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>[11]</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>[12]</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Anomaly detection using autoencoders with nonlinear dimensionality reduction</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>M. Sakurada, T. Yairi</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>MLSDA Workshop 2014</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/2689746.2689747</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[12]</t>
+          <t>[11]</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1342,162 +1342,162 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>[13]</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>Kitsune: An ensemble of autoencoders for online network intrusion detection</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>Y. Mirsky et al.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>NDSS 2018</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.14722/ndss.2018.23204</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>[14]</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>Inductive representation learning on large graphs (GraphSAGE)</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>W. Hamilton, R. Ying, J. Leskovec</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>NeurIPS 2017</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/1706.02216</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>[15]</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>Semi-supervised classification with graph convolutional networks</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>T. Kipf, M. Welling</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>ICLR 2017</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/1609.02907</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>[16]</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>PIKACHU: Temporal walk based dynamic graph embedding for network anomaly detection</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>R. Paudel, H. Huang</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>IEEE/IFIP NOMS 2022</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/noms54207.2022.9789921</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G26" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>
@@ -1622,82 +1622,82 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>[22]</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>THREATRACE: Detecting and Tracing Host-Based Threats in Node Level Through Provenance Graph Learning</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>S. Wang et al.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>IEEE TIFS 17, 2022</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2111.04333</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>[26]</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Problem space structural adversarial attacks for NIDS based on GNN classifiers</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>M. Marchetti, S. Carminati, G. Polino</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>arXiv 2024 (v1)</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2412.18218</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
@@ -1782,42 +1782,42 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>[29]</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>A unified approach to interpreting model predictions (SHAP)</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>S. Lundberg, S.-I. Lee</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>NeurIPS 2017</t>
         </is>
       </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/1705.07874</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Saharsh (A)</t>
         </is>
       </c>
     </row>
@@ -1982,122 +1982,122 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="1" t="inlineStr">
         <is>
           <t>[34]</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="1" t="inlineStr">
         <is>
           <t>Continual learning with strategic selection and forgetting (SSF)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="1" t="inlineStr">
         <is>
           <t>X. Zhang et al.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="1" t="inlineStr">
         <is>
           <t>IEEE INFOCOM 2025</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2412.16264</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="1" t="inlineStr">
         <is>
           <t>[35]</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="1" t="inlineStr">
         <is>
           <t>ReCDA: Concept drift adaptation with representation enhancement</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="1" t="inlineStr">
         <is>
           <t>S. Yang et al.</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="1" t="inlineStr">
         <is>
           <t>ACM KDD 2024</t>
         </is>
       </c>
-      <c r="F40" s="9" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3637528.3672007</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="1" t="inlineStr">
         <is>
           <t>[37]</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="1" t="inlineStr">
         <is>
           <t>Fooling LIME and SHAP</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="1" t="inlineStr">
         <is>
           <t>D. Slack et al.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="1" t="inlineStr">
         <is>
           <t>AIES 2020</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/1911.02508</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Deep (B)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
XL: Avinash locks 10 rows (2,4 + 8 new)
Assisted-by: Muse Spark (opencode)
</commit_message>
<xml_diff>
--- a/docs/report/Chapter2_40_papers.xlsx
+++ b/docs/report/Chapter2_40_papers.xlsx
@@ -862,42 +862,42 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>[1]</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Towards a taxonomy of intrusion-detection systems</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>H. Debar, M. Dacier, A. Wespi</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Comput. Networks 31(8), 1999</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/S1389-1286(98)00017-6</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
@@ -982,42 +982,42 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>[4]</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Outside the closed world: On using machine learning for network intrusion detection</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>R. Sommer, V. Paxson</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>IEEE S&amp;P 2010</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/SP.2010.25</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
@@ -1582,42 +1582,42 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>[21]</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>MAGIC: Detecting advanced persistent threats via masked graph representation learning</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Z. Jia et al.</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>USENIX Security 2024</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2310.09831</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
@@ -1702,42 +1702,42 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>[27]</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Defending network intrusion detection systems based on graph neural networks against structural adversarial attacks</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>D. Galli et al.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>IEEE NCA 2025</t>
         </is>
       </c>
-      <c r="F32" s="9" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/NCA67271.2025.00043</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
@@ -1822,162 +1822,162 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>[30]</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Real attackers don't compute gradients</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>G. Apruzzese et al.</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>IEEE SaTML 2023</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2212.14315</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>[31]</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>An adversarial robustness benchmark for enterprise network intrusion detection</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>J. Vitorino et al.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>FPS 2023</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2402.16912</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>[32]</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>TANTRA: Timing-based adversarial network traffic reshaping attack</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Y. Sharon et al.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>IEEE TIFS 17, 2022</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2103.06297</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>[33]</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Adaptative Perturbation Patterns (A2PM)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>J. Vitorino, N. Oliveira, I. Praca</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>Future Internet 14(4):108, 2022</t>
         </is>
       </c>
-      <c r="F38" s="9" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/fi14040108</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Avinash (D)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
XL: remaining 8 rows to Aditya, all 40 assigned
Assisted-by: Muse Spark (opencode)
</commit_message>
<xml_diff>
--- a/docs/report/Chapter2_40_papers.xlsx
+++ b/docs/report/Chapter2_40_papers.xlsx
@@ -1062,122 +1062,122 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>[6]</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>CSE-CIC-IDS2018 dataset</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>I. Sharafaldin et al. / Canadian Institute for Cybersecurity</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>https://www.unb.ca/cic/datasets/ids-2018.html</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>[7]</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>An empirical comparison of botnet detection methods (CTU-13)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>S. Garcia et al.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Comput. Secur. 45, 2014</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.cose.2014.05.011</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>[8]</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>UNSW-NB15: A comprehensive data set for network intrusion detection systems</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>N. Moustafa, J. Slay</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>MilCIS 2015</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/MilCIS.2015.7348942</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
@@ -1222,42 +1222,42 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>[10]</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Isolation forest</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>F. T. Liu, K. M. Ting, Z.-H. Zhou</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>ICDM 2008</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/ICDM.2008.17</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
@@ -1302,42 +1302,42 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="7" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>[11]</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Variational autoencoder based anomaly detection using reconstruction probability</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>J. An, S. Cho</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>SNU Tech. Rep. SNUDM-TR-2015-03, 2015</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>http://dm.snu.ac.kr/static/docs/TR/SNUDM-TR-2015-03.pdf</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
@@ -1502,82 +1502,82 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="7" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>[18]</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>E-GraphSAGE: A graph neural network based intrusion detection system for IoT</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>W. W. Lo et al.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>IEEE/IFIP NOMS 2022</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1109/NOMS54207.2022.9789878</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>[19]</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>Anomal-E: A self-supervised network intrusion detection system based on graph neural networks</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>E. Caville et al.</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="7" t="inlineStr">
         <is>
           <t>Knowl.-Based Syst. 258, 2022</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1016/j.knosys.2022.110030</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>
@@ -1742,42 +1742,42 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="7" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>[28]</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>A survey on concept drift adaptation</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>J. Gama et al.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>ACM Comput. Surv. 46(4), 2014</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/2523813</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Aditya (C)</t>
         </is>
       </c>
     </row>

</xml_diff>